<commit_message>
Remove 17 فهرس (lesson index) posts from article archive
These are lesson indexes (tables of contents), not written articles.
Archive reduced from 397 → 380 unique entries:
  Asdaa articles:    99
  Jeddah Club:       43
  Telegram articles: 238 (was 259, minus 17 فهرس/فهرسة posts)
  Total unique:     380

Also updated extract_articles.py to auto-exclude فهرس posts in future
runs via FIHRIS_RE pattern check on message text.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01An4PrSA3PECn9RaetfjGkW
</commit_message>
<xml_diff>
--- a/output/articles/articles_summary.xlsx
+++ b/output/articles/articles_summary.xlsx
@@ -10,8 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All (unique)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asdaa (99)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JeddahClub (43)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TGArticles (259)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duplicates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TGArticles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J398"/>
+  <dimension ref="A1:J381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17263,7 +17263,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>28.01.2026</t>
+          <t>16.02.2026</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
@@ -17273,12 +17273,12 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>فهرسة دروس لشروحات وتعليقات على #كتابالصيام |</t>
+          <t>جديدالمقالات</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>🗂️ فهرسة دروس لشروحات وتعليقات على #كتاب_الصيام | » لفضيلة الشيخ حسن بن منصور دغريري -حفظه اللّٰه ورعاه-. ➖➖➖➖🎙️ 🔻 دروس التعليق على #كتاب_الصيام من كتاب تنبيه الأنام على مافي كتاب سبل السلام من الفوائد والأحكام: •• الـــــــــ{٠١}ـــــــدرس. •• الـــــــــ{٠٢}ـــــــدرس. •• الـــ</t>
+          <t>📜 #جديد_المقالات ✿ كيف يستقبل رمضان ✿ بسم الله الرحمن الرحيم الحمد لله وحده ، والصلاة والسلام على من لا نبي بعده ، وعلى آله ، وصحبه ، ثمَّ أمَّا بعد : معاشر القراء : لقد حلَّ بابنا ضيفٌ عزيزٌ ، وشهرٌ من خير الشهور ، تظافرت بفضله الأخبار الربانية ، والنصوص الشرعية ، قال الله تعالى</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -17288,11 +17288,11 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>message6309</t>
+          <t>message6444</t>
         </is>
       </c>
       <c r="I367" t="n">
-        <v>2144</v>
+        <v>3750</v>
       </c>
       <c r="J367" t="inlineStr">
         <is>
@@ -17311,7 +17311,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>16.02.2026</t>
+          <t>22.03.2026</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
@@ -17321,12 +17321,12 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>جديدالمقالات</t>
+          <t>سائل يقول:</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>📜 #جديد_المقالات ✿ كيف يستقبل رمضان ✿ بسم الله الرحمن الرحيم الحمد لله وحده ، والصلاة والسلام على من لا نبي بعده ، وعلى آله ، وصحبه ، ثمَّ أمَّا بعد : معاشر القراء : لقد حلَّ بابنا ضيفٌ عزيزٌ ، وشهرٌ من خير الشهور ، تظافرت بفضله الأخبار الربانية ، والنصوص الشرعية ، قال الله تعالى</t>
+          <t>♦جديد♦ سائل يقول: يوجد بعض الناس ينتسبون للدعوة السلفية، لكنهم عندهم منهج تمييعي والسرورية ومعا ذالك يطعنون في أحد المشايخ في بلادناء الجزائر وهو الشيخ عبد المجيد جمعة حفظه الله تعالى الذي بين منهجهم التمييع والسرورية هل لديك علم على هذا شيخنا وما نصيحتك إلى هؤلاء شيخنا الفاضل وب</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -17336,11 +17336,11 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>message6444</t>
+          <t>message6552</t>
         </is>
       </c>
       <c r="I368" t="n">
-        <v>3750</v>
+        <v>486</v>
       </c>
       <c r="J368" t="inlineStr">
         <is>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>22.03.2026</t>
+          <t>23.03.2026</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -17374,7 +17374,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>♦جديد♦ سائل يقول: يوجد بعض الناس ينتسبون للدعوة السلفية، لكنهم عندهم منهج تمييعي والسرورية ومعا ذالك يطعنون في أحد المشايخ في بلادناء الجزائر وهو الشيخ عبد المجيد جمعة حفظه الله تعالى الذي بين منهجهم التمييع والسرورية هل لديك علم على هذا شيخنا وما نصيحتك إلى هؤلاء شيخنا الفاضل وب</t>
+          <t>♦جديد♦ سائل يقول: السلام عليكم ورحمة الله وبركاته شيخنا هناك فئة من النساء ينكرن على أخواتهن أن ينقلن أقوال العلماء التي تحذر من أهل البدع والأهواء، ويلزمنهن بالصمت وعدم الخوض في الفتن مع العلم أنهن لا يتكلمن ولا يخضن إلا بعد قراءة ردود أهل السنة على المبتدعين والمميعين والسروريي</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -17384,11 +17384,11 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>message6552</t>
+          <t>message6557</t>
         </is>
       </c>
       <c r="I369" t="n">
-        <v>486</v>
+        <v>883</v>
       </c>
       <c r="J369" t="inlineStr">
         <is>
@@ -17407,7 +17407,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>23.03.2026</t>
+          <t>04.04.2026</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
@@ -17422,7 +17422,7 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>♦جديد♦ سائل يقول: السلام عليكم ورحمة الله وبركاته شيخنا هناك فئة من النساء ينكرن على أخواتهن أن ينقلن أقوال العلماء التي تحذر من أهل البدع والأهواء، ويلزمنهن بالصمت وعدم الخوض في الفتن مع العلم أنهن لا يتكلمن ولا يخضن إلا بعد قراءة ردود أهل السنة على المبتدعين والمميعين والسروريي</t>
+          <t>#جديد 🖋 سائل يقول: أحسن الله إليكم نود منكم توضيح مسألة مهمة جدا، ألا وهي معرفة مراتب المشايخ والعلماء وتنزيلهم منازلهم اللائقة بهم. حيث يرى البعض: أن له أن يصف شيخه ويطلق ألقاب في حقه كالعلامة والجهبذ والفهامة ونحوها... من عند نفسه، دفعه لذلك حب الشيخ ودفاعه عنه. وفيه من الإخوة:</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -17432,11 +17432,11 @@
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>message6557</t>
+          <t>message6617</t>
         </is>
       </c>
       <c r="I370" t="n">
-        <v>883</v>
+        <v>758</v>
       </c>
       <c r="J370" t="inlineStr">
         <is>
@@ -17455,7 +17455,7 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>04.04.2026</t>
+          <t>25.04.2026</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
@@ -17465,12 +17465,12 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>سائل يقول:</t>
+          <t>قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله:</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>#جديد 🖋 سائل يقول: أحسن الله إليكم نود منكم توضيح مسألة مهمة جدا، ألا وهي معرفة مراتب المشايخ والعلماء وتنزيلهم منازلهم اللائقة بهم. حيث يرى البعض: أن له أن يصف شيخه ويطلق ألقاب في حقه كالعلامة والجهبذ والفهامة ونحوها... من عند نفسه، دفعه لذلك حب الشيخ ودفاعه عنه. وفيه من الإخوة:</t>
+          <t xml:space="preserve">قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله: وهل يصح أن يقول شخص أن إيمانه ، وإيمان جبريل سواء ؟ الجواب : لا يصح ، فالمرجئة يقولون الإيمان هو النطق باللسان ، والاعتقاد بالقلب ؛ والأعمال عندهم ليست من الإيمان. ونحن الآن في زمننا هذا نجد كثيراً من الناس على هذه العقيدة ، فتقول </t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
@@ -17480,15 +17480,15 @@
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>message6617</t>
+          <t>message6904</t>
         </is>
       </c>
       <c r="I371" t="n">
-        <v>758</v>
+        <v>568</v>
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>messages4.html</t>
+          <t>messages_june1.html</t>
         </is>
       </c>
     </row>
@@ -17503,7 +17503,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>25.04.2026</t>
+          <t>30.04.2026</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -17513,12 +17513,12 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله:</t>
+          <t>كتاب البيوع</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t xml:space="preserve">قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله: وهل يصح أن يقول شخص أن إيمانه ، وإيمان جبريل سواء ؟ الجواب : لا يصح ، فالمرجئة يقولون الإيمان هو النطق باللسان ، والاعتقاد بالقلب ؛ والأعمال عندهم ليست من الإيمان. ونحن الآن في زمننا هذا نجد كثيراً من الناس على هذه العقيدة ، فتقول </t>
+          <t>🔸كتاب البيوع - الدرس الأول 📎 https://t.me/daririhasan/5103 - الدرس الثاني 📎 https://t.me/daririhasan/5122 - الدرس الثالث 📎 https://t.me/daririhasan/5134 الدرس الرابع 📎 https://t.me/daririhasan/5158 - الدرس الخامس 📎 https://t.me/daririhasan/5538 - الدرس السادس 📎 https://t.me/darir</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
@@ -17528,11 +17528,11 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>message6904</t>
+          <t>message7010</t>
         </is>
       </c>
       <c r="I372" t="n">
-        <v>568</v>
+        <v>2562</v>
       </c>
       <c r="J372" t="inlineStr">
         <is>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>09.05.2026</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
@@ -17561,12 +17561,12 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>فهرس دروس معارج القبول شرح سلم الوصول للحافظ الحكمي رحمه</t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>📍فهرس دروس معارج القبول شرح سلم الوصول للحافظ الحكمي رحمه 🎙️لفضيلةالشيخ حسن الدغريري حفظه الله تعالى 📼فهـرس الدروس * ١) الدرس الأول * ⁠📎 https://t.me/daririhasan/5550 * ٢) الدرس الثاني * ⁠📎 https://t.me/daririhasan/5998 * ٣) الدرس الثالث *📎 https://t.me/daririhasan/5999 * ٤) الدر</t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وأخيراً : فهذه هي الصوفية، وهذه عقيدتها، إيمان بالمادة، وكفر بالله، إيمان بالكشف الشيطاني للشيوخ، وكفر بالقرآن، تصديق للخرافة، وجُحُودٌ للتوحيد، انغماس في البدع، ورفض للسنن، إيمان بالباطل، وكفر بالحق، تطاول عَلَى عظمة الله وألوهيته، وادعاء</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
@@ -17576,11 +17576,11 @@
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>message6971</t>
+          <t>message7162</t>
         </is>
       </c>
       <c r="I373" t="n">
-        <v>1683</v>
+        <v>576</v>
       </c>
       <c r="J373" t="inlineStr">
         <is>
@@ -17599,7 +17599,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>09.05.2026</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
@@ -17609,12 +17609,12 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>فهرس دروس شرح كتاب الفقه الميسر</t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t xml:space="preserve">📚 فهرس دروس شرح كتاب الفقه الميسر ━━━━━━━━━━━━━━━━━━━━━━ مع فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ الدرس رقم ١ 📎 [ https://t.me/daririhasan/3878 ] الدرس رقم ٢ 📎 [ https://t.me/daririhasan/307 ] الدرس رقم ٣ 📎 [ https://t.me/daririhasan/308 ] الدرس رقم ٤ 📎 [ </t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وكذلك قوله: ولا صَفَرَ »؛ فإن أهل الجاهلية كانوا يتشاءمون بشهر صفر، فأخبر النبي ﷺ أَنَّ الشهر لا شؤم فيه، بل هو كسائر الشهور، وَقَدْ كان لناس أيضا يتشاءمون ببعض الأيام كيوم الأربعاء من آخر كل شهر، ويُسمونه ربوعا لم يدور، ويعتقدون فيه أنه ي</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
@@ -17624,11 +17624,11 @@
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>message6984</t>
+          <t>message7177</t>
         </is>
       </c>
       <c r="I374" t="n">
-        <v>4141</v>
+        <v>484</v>
       </c>
       <c r="J374" t="inlineStr">
         <is>
@@ -17647,7 +17647,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>10.05.2026</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
@@ -17657,12 +17657,12 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>فهرس دروس شرح كتاب الفقه الميسر</t>
+          <t>مقال بعنوان</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>فهرس دروس شرح كتاب الفقه الميسر 2/2 الدرس رقم ٨٨ 📎 [ https://t.me/daririhasan/1541 ] الدرس رقم ٨٩ 📎 [ https://t.me/daririhasan/1548 ] الدرس رقم ٩٠ 📎 [ https://t.me/daririhasan/1576 ] الدرس رقم ٩١ 📎 [ https://t.me/daririhasan/1602 ] الدرس رقم ٩٢ 📎 [ https://t.me/daririhasan/1631 ]</t>
+          <t xml:space="preserve">مقال بعنوان الشيخ العلامة / ناصر بن أحمد جبران قحل رحمه الله ( 1361 هـ-1447هـ ) بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : أخواني القراء الفضلاء : لقد رحل صباح يوم الثلاثاء ١٨ / ١١ / ١٤٤٧ الشيخ العلامة </t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -17672,11 +17672,11 @@
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>message6985</t>
+          <t>message7186</t>
         </is>
       </c>
       <c r="I375" t="n">
-        <v>2407</v>
+        <v>3978</v>
       </c>
       <c r="J375" t="inlineStr">
         <is>
@@ -17695,7 +17695,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>10.05.2026</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
@@ -17705,12 +17705,12 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام</t>
+          <t>أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ فنظموا فيه شعراً ، وكتبوا فيه نثراً على جهده وجهاده في طلب العلم ، ونشره ، ولولا خشية الاطالة في هذا المقال لذكرت لكم بعضها ؛ وعزاؤنا في طلابه أن ينشروا علمه بين الأنام ، وسيرته الطيبة بين الناس ، ونسأل الله أن يجعل ما تركه من مقاطع صوتية نافعةٍ ، ودروس علمية مسجلة ، وتلاواتٍ قرآنية مجودة نديةٍ ، وسيرةٍ مباركةٍ مؤثرةٍ ، وعملٍ صالحٍ دلَّ عليه ، وأخلاقٍ وآدابٍ حسنةٍ تخلَّق بها ، ومريضٍ بالسحر أو غيره قد تسبب في شفائه في ميزان حسناته يوم تخف الموازين ، وأن يجمعنا به ، وبالنبيين ، والشهداء ، والصالحين ، وسائر العلماء الناصحين في جنات النعيم ، وأن يقينا جميعاً عذاب القبر والجحيم . اللهم آمين .</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>📚 فهرس دروس فتاوى أركان الإسلام ━━━━━━━━━━━━━━━━━━━━━━ 🎙 مع فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ * فتاوى_العقيدة (١) 📎 [ https://t.me/daririhasan/3544 ] * فتاوى_العقيدة (٢) 📎 [ https://t.me/daririhasan/3555 ] * فتاوى_العقيدة (٣) 📎 [ https://t.me/daririhas</t>
+          <t xml:space="preserve">أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ </t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
@@ -17720,11 +17720,11 @@
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>message6986</t>
+          <t>message7187</t>
         </is>
       </c>
       <c r="I376" t="n">
-        <v>3619</v>
+        <v>875</v>
       </c>
       <c r="J376" t="inlineStr">
         <is>
@@ -17743,7 +17743,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>11.05.2026</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
@@ -17753,12 +17753,12 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام</t>
+          <t>مقال بعنوان</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام ━━━━━━━━━━2/3 * الدرس (١) - كتاب الصلاة 📎 [ https://t.me/daririhasan/4350 ] * الدرس (٢) - كتاب الصلاة 📎 [ https://t.me/daririhasan/4352 ] * الدرس (٣) - كتاب الصلاة 📎 [ https://t.me/daririhasan/4366 ] * الدرس (٤) - كتاب الصلاة 📎 [ https://t.me/daririh</t>
+          <t>مقال بعنوان الذكاء الاصطناعي ، ومواقع التواصل الاجتماعي بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : معاشر القراء الكرام : إنَّ نعمة الجوالات الحديثة ، وأجهزة الحاسب الآلي نعمةٌ عظيمة إذا استخدمت فيما ينف</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
@@ -17768,11 +17768,11 @@
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>message6987</t>
+          <t>message7200</t>
         </is>
       </c>
       <c r="I377" t="n">
-        <v>4193</v>
+        <v>4081</v>
       </c>
       <c r="J377" t="inlineStr">
         <is>
@@ -17791,7 +17791,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>11.05.2026</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
@@ -17801,12 +17801,12 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام</t>
+          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِنْدَ اللَّهِ عَظِيمٌ – النور : 15 وقال صلى الله عليه وسلـم : – كَفَى بِالْمَرْءِ كَذِبًا أَنْ يُحَدِّثَ بِكُلِّ مَا سمع – رَوَاهُ مُسلم ؛ نسأل الله أن يديم علينا نعمه الظاهرة والباطنة ، وأن يوزعنا ذكرها وشكرها ، ومنها نعمة الجوالات والحاسوبات ، وما فيها من برامج ؛ وتقنيات نافعةٍ ؛ لخدمة الدين ، ثمَّ المليك ، والوطن .</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t xml:space="preserve">فهرس دروس فتاوى أركان الإسلام 3/3 * الدرس (٦٧) - كتاب الصلاة 📎 [ https://t.me/daririhasan/5499 ] * الدرس (٦٨) - كتاب الصلاة 📎 [ https://t.me/daririhasan/5511 ] * الدرس (١) - كتاب الحج 📎 [ https://t.me/daririhasan/4410 ] * الدرس (٢) - كتاب الحج 📎 [ https://t.me/daririhasan/4422 ] </t>
+          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِن</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
@@ -17816,11 +17816,11 @@
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>message6988</t>
+          <t>message7201</t>
         </is>
       </c>
       <c r="I378" t="n">
-        <v>1439</v>
+        <v>1062</v>
       </c>
       <c r="J378" t="inlineStr">
         <is>
@@ -17839,7 +17839,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>15.04.2026</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
@@ -17849,12 +17849,12 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>فهرس دروس القول السديد شرح كتاب التوحيد</t>
+          <t>جديد 💥</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>📚 فهرس دروس القول السديد شرح كتاب التوحيد ━━━━━━━━━━━━━━━━━━━━━━ 🎙 مع فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ ━━━━━━━━━━━━━━━━━━━━━━ الدرس رقم ١ 📎 [ https://t.me/daririhasan/4678 ] الدرس رقم ٢ 📎 https://t.me/daririhasan/4709 ] الدرس رقم ٣ 📎 [ https://t.me/da</t>
+          <t xml:space="preserve">💥جديد 💥 📖 { العِلْمُ أشْرَفُ مَطْلُوبٍ وَطَالِبُهُ للهِ أكْرَمُ مَن يَمْشِي عَلى قَدَمِ } 📚 🎙️( تم التسجيل- بحمدالله تعالى )🔊 📌 [ الدروس العلمية ]📚 📌" لشهر- شوال " 1447/10/26هجري 🌱 📋 " اسبوعياً " كل يوم الثلاثاء ✅ 🕣 بعد صلاة العشاء👇 📡《عن بُعد 》📡 📚 شرح كتاب- [ معارج القبول في شرح </t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
@@ -17864,15 +17864,15 @@
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>message6989</t>
+          <t>message6787</t>
         </is>
       </c>
       <c r="I379" t="n">
-        <v>777</v>
+        <v>772</v>
       </c>
       <c r="J379" t="inlineStr">
         <is>
-          <t>messages_june1.html</t>
+          <t>messages_new.html</t>
         </is>
       </c>
     </row>
@@ -17887,7 +17887,7 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>17.04.2026</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
@@ -17897,12 +17897,12 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>فهرس خطبة الجمعة</t>
+          <t>ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!»</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 1 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ١) صفة صلاة النبي ﷺ | ٢٤ جمادى الآخرة ١٤٣٨هـ 📎 https://t.me/daririhasan/80 ٢) سيرة الإمام زيد بن محمد المدخلي | ٢٤ جمادى الآخرة ١٤٣٨هـ 📎 https://t.me/daririhas</t>
+          <t>#فوائد ♦|«ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله- : «وإنَّ ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة، والاستهانة بهم؛ لأن هذا ممَّا يُس</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
@@ -17912,15 +17912,15 @@
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>message6999</t>
+          <t>message6817</t>
         </is>
       </c>
       <c r="I380" t="n">
-        <v>4015</v>
+        <v>936</v>
       </c>
       <c r="J380" t="inlineStr">
         <is>
-          <t>messages_june1.html</t>
+          <t>messages_new.html</t>
         </is>
       </c>
     </row>
@@ -17935,7 +17935,7 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>17.04.2026</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
@@ -17945,12 +17945,12 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>فهرس خطبة الجمعة</t>
+          <t>يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!»</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t xml:space="preserve">📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 2 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٥١) من أحكام النكاح ٢ | ١٥ ربيع الأول ١٤٤١هـ 📎 https://t.me/daririhasan/496 ٥٢) من أحكام النكاح ٣ | ١٥ ربيع الأول ١٤٤١هـ 📎 https://t.me/daririhasan/497 ٥٣) من </t>
+          <t xml:space="preserve">#فوائد ♦|«يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله-: «فالمهم أنَّ الدعوة يبدأ فيها بالأهم فالمهم، وأنَّ الدعوة إلى التوحيد لمن أهم المهمات؛ يجب عليك أن تُنصِّص على </t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -17960,829 +17960,13 @@
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>message7000</t>
+          <t>message6820</t>
         </is>
       </c>
       <c r="I381" t="n">
-        <v>4026</v>
+        <v>1318</v>
       </c>
       <c r="J381" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" t="n">
-        <v>381</v>
-      </c>
-      <c r="B382" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C382" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D382" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E382" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F382" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 3 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٩٨) جماعة الإخوان المسلمين | ٦ ربيع الثاني ١٤٤٢هـ 📎 https://t.me/daririhasan/1301 ٩٩) رزق الله تعالى لعباده | ١٢ ربيع الثاني ١٤٤٢هـ 📎 https://t.me/daririhasan/</t>
-        </is>
-      </c>
-      <c r="G382" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H382" t="inlineStr">
-        <is>
-          <t>message7001</t>
-        </is>
-      </c>
-      <c r="I382" t="n">
-        <v>4034</v>
-      </c>
-      <c r="J382" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" t="n">
-        <v>382</v>
-      </c>
-      <c r="B383" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C383" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D383" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E383" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F383" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 4 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ١٤٥) عبد الرحمن بن عوف رضي الله عنه | ٢٠ ذو الحجة ١٤٤٢هـ 📎 https://t.me/daririhasan/1690 ١٤٦) نهاية العام والأخذ بالاحترازات ضد كورونا | ٢٧ ذو الحجة ١٤٤٢هـ 📎 h</t>
-        </is>
-      </c>
-      <c r="G383" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H383" t="inlineStr">
-        <is>
-          <t>message7002</t>
-        </is>
-      </c>
-      <c r="I383" t="n">
-        <v>4014</v>
-      </c>
-      <c r="J383" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" t="n">
-        <v>383</v>
-      </c>
-      <c r="B384" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C384" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D384" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E384" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F384" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 5 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ١٩١) من أحكام الأضحية | ٥ ذو الحجة ١٤٤٣هـ 📎 https://t.me/daririhasan/2280 ١٩٢) أفضل أيام العام | ٩ ذو الحجة ١٤٤٣هـ 📎 https://t.me/daririhasan/2288 ١٩٣) المدينة</t>
-        </is>
-      </c>
-      <c r="G384" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H384" t="inlineStr">
-        <is>
-          <t>message7003</t>
-        </is>
-      </c>
-      <c r="I384" t="n">
-        <v>4019</v>
-      </c>
-      <c r="J384" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="385">
-      <c r="A385" t="n">
-        <v>384</v>
-      </c>
-      <c r="B385" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C385" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D385" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E385" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F385" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 6 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٢٣٦) قصة موسى عليه السلام (٧) | ٦ ذو القعدة ١٤٤٤هـ 📎 https://t.me/daririhasan/3328 ٢٣٧) قصة موسى عليه السلام (٨) | ١٣ ذو القعدة ١٤٤٤هـ 📎 https://t.me/daririhas</t>
-        </is>
-      </c>
-      <c r="G385" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H385" t="inlineStr">
-        <is>
-          <t>message7004</t>
-        </is>
-      </c>
-      <c r="I385" t="n">
-        <v>3953</v>
-      </c>
-      <c r="J385" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" t="n">
-        <v>385</v>
-      </c>
-      <c r="B386" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C386" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D386" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E386" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F386" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 7 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٢٨٢) الأعمال الصالحة في العشر والأخذ بأسباب السلامة في الحج | ١ ذو الحجة ١٤٤٥هـ 📎 https://t.me/daririhasan/4449 ٢٨٣) صفة الأنساك الثلاثة (٢) | ١٢ ذو الحجة ١٤٤٥</t>
-        </is>
-      </c>
-      <c r="G386" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H386" t="inlineStr">
-        <is>
-          <t>message7005</t>
-        </is>
-      </c>
-      <c r="I386" t="n">
-        <v>3958</v>
-      </c>
-      <c r="J386" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="387">
-      <c r="A387" t="n">
-        <v>386</v>
-      </c>
-      <c r="B387" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C387" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D387" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E387" t="inlineStr">
-        <is>
-          <t>فهرس دروس الأفنان الندية شرح السبل السوية في فقه السنن المروية للشيخ العلامة زيد المدخلي رحمه الله</t>
-        </is>
-      </c>
-      <c r="F387" t="inlineStr">
-        <is>
-          <t>📍فهرس دروس الأفنان الندية شرح السبل السوية في فقه السنن المروية للشيخ العلامة زيد المدخلي رحمه الله 🎙️لفضيلة الشيخ حسن الدغريري حفظه الله 🔹فهرس الدروس : 🔸 كتاب الطهارة - الدرس الأول 📎 https://t.me/daririhasan/2371 - الدرس الثاني 📎 https://t.me/daririhasan/2392 - الدرس الثالث 📎 ht</t>
-        </is>
-      </c>
-      <c r="G387" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H387" t="inlineStr">
-        <is>
-          <t>message7008</t>
-        </is>
-      </c>
-      <c r="I387" t="n">
-        <v>4062</v>
-      </c>
-      <c r="J387" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="388">
-      <c r="A388" t="n">
-        <v>387</v>
-      </c>
-      <c r="B388" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C388" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D388" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E388" t="inlineStr">
-        <is>
-          <t>كتاب البيوع</t>
-        </is>
-      </c>
-      <c r="F388" t="inlineStr">
-        <is>
-          <t>🔸كتاب البيوع - الدرس الأول 📎 https://t.me/daririhasan/5103 - الدرس الثاني 📎 https://t.me/daririhasan/5122 - الدرس الثالث 📎 https://t.me/daririhasan/5134 الدرس الرابع 📎 https://t.me/daririhasan/5158 - الدرس الخامس 📎 https://t.me/daririhasan/5538 - الدرس السادس 📎 https://t.me/darir</t>
-        </is>
-      </c>
-      <c r="G388" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H388" t="inlineStr">
-        <is>
-          <t>message7010</t>
-        </is>
-      </c>
-      <c r="I388" t="n">
-        <v>2562</v>
-      </c>
-      <c r="J388" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="389">
-      <c r="A389" t="n">
-        <v>388</v>
-      </c>
-      <c r="B389" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C389" t="inlineStr">
-        <is>
-          <t>09.05.2026</t>
-        </is>
-      </c>
-      <c r="D389" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E389" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
-        </is>
-      </c>
-      <c r="F389" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وأخيراً : فهذه هي الصوفية، وهذه عقيدتها، إيمان بالمادة، وكفر بالله، إيمان بالكشف الشيطاني للشيوخ، وكفر بالقرآن، تصديق للخرافة، وجُحُودٌ للتوحيد، انغماس في البدع، ورفض للسنن، إيمان بالباطل، وكفر بالحق، تطاول عَلَى عظمة الله وألوهيته، وادعاء</t>
-        </is>
-      </c>
-      <c r="G389" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H389" t="inlineStr">
-        <is>
-          <t>message7162</t>
-        </is>
-      </c>
-      <c r="I389" t="n">
-        <v>576</v>
-      </c>
-      <c r="J389" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="390">
-      <c r="A390" t="n">
-        <v>389</v>
-      </c>
-      <c r="B390" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C390" t="inlineStr">
-        <is>
-          <t>09.05.2026</t>
-        </is>
-      </c>
-      <c r="D390" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E390" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
-        </is>
-      </c>
-      <c r="F390" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وكذلك قوله: ولا صَفَرَ »؛ فإن أهل الجاهلية كانوا يتشاءمون بشهر صفر، فأخبر النبي ﷺ أَنَّ الشهر لا شؤم فيه، بل هو كسائر الشهور، وَقَدْ كان لناس أيضا يتشاءمون ببعض الأيام كيوم الأربعاء من آخر كل شهر، ويُسمونه ربوعا لم يدور، ويعتقدون فيه أنه ي</t>
-        </is>
-      </c>
-      <c r="G390" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H390" t="inlineStr">
-        <is>
-          <t>message7177</t>
-        </is>
-      </c>
-      <c r="I390" t="n">
-        <v>484</v>
-      </c>
-      <c r="J390" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="391">
-      <c r="A391" t="n">
-        <v>390</v>
-      </c>
-      <c r="B391" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C391" t="inlineStr">
-        <is>
-          <t>10.05.2026</t>
-        </is>
-      </c>
-      <c r="D391" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E391" t="inlineStr">
-        <is>
-          <t>مقال بعنوان</t>
-        </is>
-      </c>
-      <c r="F391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مقال بعنوان الشيخ العلامة / ناصر بن أحمد جبران قحل رحمه الله ( 1361 هـ-1447هـ ) بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : أخواني القراء الفضلاء : لقد رحل صباح يوم الثلاثاء ١٨ / ١١ / ١٤٤٧ الشيخ العلامة </t>
-        </is>
-      </c>
-      <c r="G391" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H391" t="inlineStr">
-        <is>
-          <t>message7186</t>
-        </is>
-      </c>
-      <c r="I391" t="n">
-        <v>3978</v>
-      </c>
-      <c r="J391" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="392">
-      <c r="A392" t="n">
-        <v>391</v>
-      </c>
-      <c r="B392" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C392" t="inlineStr">
-        <is>
-          <t>10.05.2026</t>
-        </is>
-      </c>
-      <c r="D392" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E392" t="inlineStr">
-        <is>
-          <t>أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ فنظموا فيه شعراً ، وكتبوا فيه نثراً على جهده وجهاده في طلب العلم ، ونشره ، ولولا خشية الاطالة في هذا المقال لذكرت لكم بعضها ؛ وعزاؤنا في طلابه أن ينشروا علمه بين الأنام ، وسيرته الطيبة بين الناس ، ونسأل الله أن يجعل ما تركه من مقاطع صوتية نافعةٍ ، ودروس علمية مسجلة ، وتلاواتٍ قرآنية مجودة نديةٍ ، وسيرةٍ مباركةٍ مؤثرةٍ ، وعملٍ صالحٍ دلَّ عليه ، وأخلاقٍ وآدابٍ حسنةٍ تخلَّق بها ، ومريضٍ بالسحر أو غيره قد تسبب في شفائه في ميزان حسناته يوم تخف الموازين ، وأن يجمعنا به ، وبالنبيين ، والشهداء ، والصالحين ، وسائر العلماء الناصحين في جنات النعيم ، وأن يقينا جميعاً عذاب القبر والجحيم . اللهم آمين .</t>
-        </is>
-      </c>
-      <c r="F392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ </t>
-        </is>
-      </c>
-      <c r="G392" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H392" t="inlineStr">
-        <is>
-          <t>message7187</t>
-        </is>
-      </c>
-      <c r="I392" t="n">
-        <v>875</v>
-      </c>
-      <c r="J392" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="393">
-      <c r="A393" t="n">
-        <v>392</v>
-      </c>
-      <c r="B393" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C393" t="inlineStr">
-        <is>
-          <t>11.05.2026</t>
-        </is>
-      </c>
-      <c r="D393" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E393" t="inlineStr">
-        <is>
-          <t>مقال بعنوان</t>
-        </is>
-      </c>
-      <c r="F393" t="inlineStr">
-        <is>
-          <t>مقال بعنوان الذكاء الاصطناعي ، ومواقع التواصل الاجتماعي بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : معاشر القراء الكرام : إنَّ نعمة الجوالات الحديثة ، وأجهزة الحاسب الآلي نعمةٌ عظيمة إذا استخدمت فيما ينف</t>
-        </is>
-      </c>
-      <c r="G393" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H393" t="inlineStr">
-        <is>
-          <t>message7200</t>
-        </is>
-      </c>
-      <c r="I393" t="n">
-        <v>4081</v>
-      </c>
-      <c r="J393" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="394">
-      <c r="A394" t="n">
-        <v>393</v>
-      </c>
-      <c r="B394" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C394" t="inlineStr">
-        <is>
-          <t>11.05.2026</t>
-        </is>
-      </c>
-      <c r="D394" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E394" t="inlineStr">
-        <is>
-          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِنْدَ اللَّهِ عَظِيمٌ – النور : 15 وقال صلى الله عليه وسلـم : – كَفَى بِالْمَرْءِ كَذِبًا أَنْ يُحَدِّثَ بِكُلِّ مَا سمع – رَوَاهُ مُسلم ؛ نسأل الله أن يديم علينا نعمه الظاهرة والباطنة ، وأن يوزعنا ذكرها وشكرها ، ومنها نعمة الجوالات والحاسوبات ، وما فيها من برامج ؛ وتقنيات نافعةٍ ؛ لخدمة الدين ، ثمَّ المليك ، والوطن .</t>
-        </is>
-      </c>
-      <c r="F394" t="inlineStr">
-        <is>
-          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِن</t>
-        </is>
-      </c>
-      <c r="G394" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H394" t="inlineStr">
-        <is>
-          <t>message7201</t>
-        </is>
-      </c>
-      <c r="I394" t="n">
-        <v>1062</v>
-      </c>
-      <c r="J394" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="395">
-      <c r="A395" t="n">
-        <v>394</v>
-      </c>
-      <c r="B395" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C395" t="inlineStr">
-        <is>
-          <t>21.05.2026</t>
-        </is>
-      </c>
-      <c r="D395" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E395" t="inlineStr">
-        <is>
-          <t>فهرس دروس</t>
-        </is>
-      </c>
-      <c r="F395" t="inlineStr">
-        <is>
-          <t>فهرس دروس #التعليق_على_كتاب_الأربعين_النووية 🎙 للشيخ الفاضل: #حسن_بن_محمد_الدغريري -الدرس الأول 📎 https://t.me/daririhasan/705 -الدرس الثاني 📎 https://t.me/daririhasan/708 -الدرس الثالث 📎 https://t.me/daririhasan/709 -الدرس الرابع 📎 https://t.me/daririhasan/717 -الدرس الخامس 📎 ht</t>
-        </is>
-      </c>
-      <c r="G395" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H395" t="inlineStr">
-        <is>
-          <t>message7423</t>
-        </is>
-      </c>
-      <c r="I395" t="n">
-        <v>2391</v>
-      </c>
-      <c r="J395" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="396">
-      <c r="A396" t="n">
-        <v>395</v>
-      </c>
-      <c r="B396" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C396" t="inlineStr">
-        <is>
-          <t>15.04.2026</t>
-        </is>
-      </c>
-      <c r="D396" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E396" t="inlineStr">
-        <is>
-          <t>جديد 💥</t>
-        </is>
-      </c>
-      <c r="F396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">💥جديد 💥 📖 { العِلْمُ أشْرَفُ مَطْلُوبٍ وَطَالِبُهُ للهِ أكْرَمُ مَن يَمْشِي عَلى قَدَمِ } 📚 🎙️( تم التسجيل- بحمدالله تعالى )🔊 📌 [ الدروس العلمية ]📚 📌" لشهر- شوال " 1447/10/26هجري 🌱 📋 " اسبوعياً " كل يوم الثلاثاء ✅ 🕣 بعد صلاة العشاء👇 📡《عن بُعد 》📡 📚 شرح كتاب- [ معارج القبول في شرح </t>
-        </is>
-      </c>
-      <c r="G396" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H396" t="inlineStr">
-        <is>
-          <t>message6787</t>
-        </is>
-      </c>
-      <c r="I396" t="n">
-        <v>772</v>
-      </c>
-      <c r="J396" t="inlineStr">
-        <is>
-          <t>messages_new.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="397">
-      <c r="A397" t="n">
-        <v>396</v>
-      </c>
-      <c r="B397" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C397" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
-      </c>
-      <c r="D397" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E397" t="inlineStr">
-        <is>
-          <t>ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!»</t>
-        </is>
-      </c>
-      <c r="F397" t="inlineStr">
-        <is>
-          <t>#فوائد ♦|«ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله- : «وإنَّ ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة، والاستهانة بهم؛ لأن هذا ممَّا يُس</t>
-        </is>
-      </c>
-      <c r="G397" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H397" t="inlineStr">
-        <is>
-          <t>message6817</t>
-        </is>
-      </c>
-      <c r="I397" t="n">
-        <v>936</v>
-      </c>
-      <c r="J397" t="inlineStr">
-        <is>
-          <t>messages_new.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="398">
-      <c r="A398" t="n">
-        <v>397</v>
-      </c>
-      <c r="B398" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C398" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
-      </c>
-      <c r="D398" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E398" t="inlineStr">
-        <is>
-          <t>يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!»</t>
-        </is>
-      </c>
-      <c r="F398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#فوائد ♦|«يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله-: «فالمهم أنَّ الدعوة يبدأ فيها بالأهم فالمهم، وأنَّ الدعوة إلى التوحيد لمن أهم المهمات؛ يجب عليك أن تُنصِّص على </t>
-        </is>
-      </c>
-      <c r="G398" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H398" t="inlineStr">
-        <is>
-          <t>message6820</t>
-        </is>
-      </c>
-      <c r="I398" t="n">
-        <v>1318</v>
-      </c>
-      <c r="J398" t="inlineStr">
         <is>
           <t>messages_new.html</t>
         </is>
@@ -25007,7 +24191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J256"/>
+  <dimension ref="A1:J239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35777,7 +34961,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>28.01.2026</t>
+          <t>16.02.2026</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -35787,12 +34971,12 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>فهرسة دروس لشروحات وتعليقات على #كتابالصيام |</t>
+          <t>جديدالمقالات</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>🗂️ فهرسة دروس لشروحات وتعليقات على #كتاب_الصيام | » لفضيلة الشيخ حسن بن منصور دغريري -حفظه اللّٰه ورعاه-. ➖➖➖➖🎙️ 🔻 دروس التعليق على #كتاب_الصيام من كتاب تنبيه الأنام على مافي كتاب سبل السلام من الفوائد والأحكام: •• الـــــــــ{٠١}ـــــــدرس. •• الـــــــــ{٠٢}ـــــــدرس. •• الـــ</t>
+          <t>📜 #جديد_المقالات ✿ كيف يستقبل رمضان ✿ بسم الله الرحمن الرحيم الحمد لله وحده ، والصلاة والسلام على من لا نبي بعده ، وعلى آله ، وصحبه ، ثمَّ أمَّا بعد : معاشر القراء : لقد حلَّ بابنا ضيفٌ عزيزٌ ، وشهرٌ من خير الشهور ، تظافرت بفضله الأخبار الربانية ، والنصوص الشرعية ، قال الله تعالى</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -35802,11 +34986,11 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>message6309</t>
+          <t>message6444</t>
         </is>
       </c>
       <c r="I225" t="n">
-        <v>2144</v>
+        <v>3750</v>
       </c>
       <c r="J225" t="inlineStr">
         <is>
@@ -35825,7 +35009,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16.02.2026</t>
+          <t>22.03.2026</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -35835,12 +35019,12 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>جديدالمقالات</t>
+          <t>سائل يقول:</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>📜 #جديد_المقالات ✿ كيف يستقبل رمضان ✿ بسم الله الرحمن الرحيم الحمد لله وحده ، والصلاة والسلام على من لا نبي بعده ، وعلى آله ، وصحبه ، ثمَّ أمَّا بعد : معاشر القراء : لقد حلَّ بابنا ضيفٌ عزيزٌ ، وشهرٌ من خير الشهور ، تظافرت بفضله الأخبار الربانية ، والنصوص الشرعية ، قال الله تعالى</t>
+          <t>♦جديد♦ سائل يقول: يوجد بعض الناس ينتسبون للدعوة السلفية، لكنهم عندهم منهج تمييعي والسرورية ومعا ذالك يطعنون في أحد المشايخ في بلادناء الجزائر وهو الشيخ عبد المجيد جمعة حفظه الله تعالى الذي بين منهجهم التمييع والسرورية هل لديك علم على هذا شيخنا وما نصيحتك إلى هؤلاء شيخنا الفاضل وب</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -35850,11 +35034,11 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>message6444</t>
+          <t>message6552</t>
         </is>
       </c>
       <c r="I226" t="n">
-        <v>3750</v>
+        <v>486</v>
       </c>
       <c r="J226" t="inlineStr">
         <is>
@@ -35873,7 +35057,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>22.03.2026</t>
+          <t>23.03.2026</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -35888,7 +35072,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>♦جديد♦ سائل يقول: يوجد بعض الناس ينتسبون للدعوة السلفية، لكنهم عندهم منهج تمييعي والسرورية ومعا ذالك يطعنون في أحد المشايخ في بلادناء الجزائر وهو الشيخ عبد المجيد جمعة حفظه الله تعالى الذي بين منهجهم التمييع والسرورية هل لديك علم على هذا شيخنا وما نصيحتك إلى هؤلاء شيخنا الفاضل وب</t>
+          <t>♦جديد♦ سائل يقول: السلام عليكم ورحمة الله وبركاته شيخنا هناك فئة من النساء ينكرن على أخواتهن أن ينقلن أقوال العلماء التي تحذر من أهل البدع والأهواء، ويلزمنهن بالصمت وعدم الخوض في الفتن مع العلم أنهن لا يتكلمن ولا يخضن إلا بعد قراءة ردود أهل السنة على المبتدعين والمميعين والسروريي</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -35898,11 +35082,11 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>message6552</t>
+          <t>message6557</t>
         </is>
       </c>
       <c r="I227" t="n">
-        <v>486</v>
+        <v>883</v>
       </c>
       <c r="J227" t="inlineStr">
         <is>
@@ -35921,7 +35105,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>23.03.2026</t>
+          <t>04.04.2026</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -35936,7 +35120,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>♦جديد♦ سائل يقول: السلام عليكم ورحمة الله وبركاته شيخنا هناك فئة من النساء ينكرن على أخواتهن أن ينقلن أقوال العلماء التي تحذر من أهل البدع والأهواء، ويلزمنهن بالصمت وعدم الخوض في الفتن مع العلم أنهن لا يتكلمن ولا يخضن إلا بعد قراءة ردود أهل السنة على المبتدعين والمميعين والسروريي</t>
+          <t>#جديد 🖋 سائل يقول: أحسن الله إليكم نود منكم توضيح مسألة مهمة جدا، ألا وهي معرفة مراتب المشايخ والعلماء وتنزيلهم منازلهم اللائقة بهم. حيث يرى البعض: أن له أن يصف شيخه ويطلق ألقاب في حقه كالعلامة والجهبذ والفهامة ونحوها... من عند نفسه، دفعه لذلك حب الشيخ ودفاعه عنه. وفيه من الإخوة:</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -35946,11 +35130,11 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>message6557</t>
+          <t>message6617</t>
         </is>
       </c>
       <c r="I228" t="n">
-        <v>883</v>
+        <v>758</v>
       </c>
       <c r="J228" t="inlineStr">
         <is>
@@ -35969,7 +35153,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>04.04.2026</t>
+          <t>25.04.2026</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -35979,12 +35163,12 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>سائل يقول:</t>
+          <t>قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله:</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>#جديد 🖋 سائل يقول: أحسن الله إليكم نود منكم توضيح مسألة مهمة جدا، ألا وهي معرفة مراتب المشايخ والعلماء وتنزيلهم منازلهم اللائقة بهم. حيث يرى البعض: أن له أن يصف شيخه ويطلق ألقاب في حقه كالعلامة والجهبذ والفهامة ونحوها... من عند نفسه، دفعه لذلك حب الشيخ ودفاعه عنه. وفيه من الإخوة:</t>
+          <t xml:space="preserve">قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله: وهل يصح أن يقول شخص أن إيمانه ، وإيمان جبريل سواء ؟ الجواب : لا يصح ، فالمرجئة يقولون الإيمان هو النطق باللسان ، والاعتقاد بالقلب ؛ والأعمال عندهم ليست من الإيمان. ونحن الآن في زمننا هذا نجد كثيراً من الناس على هذه العقيدة ، فتقول </t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -35994,15 +35178,15 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>message6617</t>
+          <t>message6904</t>
         </is>
       </c>
       <c r="I229" t="n">
-        <v>758</v>
+        <v>568</v>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>messages4.html</t>
+          <t>messages_june1.html</t>
         </is>
       </c>
     </row>
@@ -36017,7 +35201,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>25.04.2026</t>
+          <t>30.04.2026</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -36027,12 +35211,12 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله:</t>
+          <t>كتاب البيوع</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t xml:space="preserve">قال الشيخ العلامة أحمد بن يحيى النجمي رحمه الله: وهل يصح أن يقول شخص أن إيمانه ، وإيمان جبريل سواء ؟ الجواب : لا يصح ، فالمرجئة يقولون الإيمان هو النطق باللسان ، والاعتقاد بالقلب ؛ والأعمال عندهم ليست من الإيمان. ونحن الآن في زمننا هذا نجد كثيراً من الناس على هذه العقيدة ، فتقول </t>
+          <t>🔸كتاب البيوع - الدرس الأول 📎 https://t.me/daririhasan/5103 - الدرس الثاني 📎 https://t.me/daririhasan/5122 - الدرس الثالث 📎 https://t.me/daririhasan/5134 الدرس الرابع 📎 https://t.me/daririhasan/5158 - الدرس الخامس 📎 https://t.me/daririhasan/5538 - الدرس السادس 📎 https://t.me/darir</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -36042,11 +35226,11 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>message6904</t>
+          <t>message7010</t>
         </is>
       </c>
       <c r="I230" t="n">
-        <v>568</v>
+        <v>2562</v>
       </c>
       <c r="J230" t="inlineStr">
         <is>
@@ -36065,7 +35249,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>09.05.2026</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -36075,12 +35259,12 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>فهرس دروس معارج القبول شرح سلم الوصول للحافظ الحكمي رحمه</t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>📍فهرس دروس معارج القبول شرح سلم الوصول للحافظ الحكمي رحمه 🎙️لفضيلةالشيخ حسن الدغريري حفظه الله تعالى 📼فهـرس الدروس * ١) الدرس الأول * ⁠📎 https://t.me/daririhasan/5550 * ٢) الدرس الثاني * ⁠📎 https://t.me/daririhasan/5998 * ٣) الدرس الثالث *📎 https://t.me/daririhasan/5999 * ٤) الدر</t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وأخيراً : فهذه هي الصوفية، وهذه عقيدتها، إيمان بالمادة، وكفر بالله، إيمان بالكشف الشيطاني للشيوخ، وكفر بالقرآن، تصديق للخرافة، وجُحُودٌ للتوحيد، انغماس في البدع، ورفض للسنن، إيمان بالباطل، وكفر بالحق، تطاول عَلَى عظمة الله وألوهيته، وادعاء</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -36090,11 +35274,11 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>message6971</t>
+          <t>message7162</t>
         </is>
       </c>
       <c r="I231" t="n">
-        <v>1683</v>
+        <v>576</v>
       </c>
       <c r="J231" t="inlineStr">
         <is>
@@ -36113,7 +35297,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>09.05.2026</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -36123,12 +35307,12 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>فهرس دروس شرح كتاب الفقه الميسر</t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t xml:space="preserve">📚 فهرس دروس شرح كتاب الفقه الميسر ━━━━━━━━━━━━━━━━━━━━━━ مع فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ الدرس رقم ١ 📎 [ https://t.me/daririhasan/3878 ] الدرس رقم ٢ 📎 [ https://t.me/daririhasan/307 ] الدرس رقم ٣ 📎 [ https://t.me/daririhasan/308 ] الدرس رقم ٤ 📎 [ </t>
+          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وكذلك قوله: ولا صَفَرَ »؛ فإن أهل الجاهلية كانوا يتشاءمون بشهر صفر، فأخبر النبي ﷺ أَنَّ الشهر لا شؤم فيه، بل هو كسائر الشهور، وَقَدْ كان لناس أيضا يتشاءمون ببعض الأيام كيوم الأربعاء من آخر كل شهر، ويُسمونه ربوعا لم يدور، ويعتقدون فيه أنه ي</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -36138,11 +35322,11 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>message6984</t>
+          <t>message7177</t>
         </is>
       </c>
       <c r="I232" t="n">
-        <v>4141</v>
+        <v>484</v>
       </c>
       <c r="J232" t="inlineStr">
         <is>
@@ -36161,7 +35345,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>10.05.2026</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -36171,12 +35355,12 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>فهرس دروس شرح كتاب الفقه الميسر</t>
+          <t>مقال بعنوان</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>فهرس دروس شرح كتاب الفقه الميسر 2/2 الدرس رقم ٨٨ 📎 [ https://t.me/daririhasan/1541 ] الدرس رقم ٨٩ 📎 [ https://t.me/daririhasan/1548 ] الدرس رقم ٩٠ 📎 [ https://t.me/daririhasan/1576 ] الدرس رقم ٩١ 📎 [ https://t.me/daririhasan/1602 ] الدرس رقم ٩٢ 📎 [ https://t.me/daririhasan/1631 ]</t>
+          <t xml:space="preserve">مقال بعنوان الشيخ العلامة / ناصر بن أحمد جبران قحل رحمه الله ( 1361 هـ-1447هـ ) بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : أخواني القراء الفضلاء : لقد رحل صباح يوم الثلاثاء ١٨ / ١١ / ١٤٤٧ الشيخ العلامة </t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -36186,11 +35370,11 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>message6985</t>
+          <t>message7186</t>
         </is>
       </c>
       <c r="I233" t="n">
-        <v>2407</v>
+        <v>3978</v>
       </c>
       <c r="J233" t="inlineStr">
         <is>
@@ -36209,7 +35393,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>10.05.2026</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -36219,12 +35403,12 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام</t>
+          <t>أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ فنظموا فيه شعراً ، وكتبوا فيه نثراً على جهده وجهاده في طلب العلم ، ونشره ، ولولا خشية الاطالة في هذا المقال لذكرت لكم بعضها ؛ وعزاؤنا في طلابه أن ينشروا علمه بين الأنام ، وسيرته الطيبة بين الناس ، ونسأل الله أن يجعل ما تركه من مقاطع صوتية نافعةٍ ، ودروس علمية مسجلة ، وتلاواتٍ قرآنية مجودة نديةٍ ، وسيرةٍ مباركةٍ مؤثرةٍ ، وعملٍ صالحٍ دلَّ عليه ، وأخلاقٍ وآدابٍ حسنةٍ تخلَّق بها ، ومريضٍ بالسحر أو غيره قد تسبب في شفائه في ميزان حسناته يوم تخف الموازين ، وأن يجمعنا به ، وبالنبيين ، والشهداء ، والصالحين ، وسائر العلماء الناصحين في جنات النعيم ، وأن يقينا جميعاً عذاب القبر والجحيم . اللهم آمين .</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>📚 فهرس دروس فتاوى أركان الإسلام ━━━━━━━━━━━━━━━━━━━━━━ 🎙 مع فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ * فتاوى_العقيدة (١) 📎 [ https://t.me/daririhasan/3544 ] * فتاوى_العقيدة (٢) 📎 [ https://t.me/daririhasan/3555 ] * فتاوى_العقيدة (٣) 📎 [ https://t.me/daririhas</t>
+          <t xml:space="preserve">أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ </t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -36234,11 +35418,11 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>message6986</t>
+          <t>message7187</t>
         </is>
       </c>
       <c r="I234" t="n">
-        <v>3619</v>
+        <v>875</v>
       </c>
       <c r="J234" t="inlineStr">
         <is>
@@ -36257,7 +35441,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>11.05.2026</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -36267,12 +35451,12 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام</t>
+          <t>مقال بعنوان</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام ━━━━━━━━━━2/3 * الدرس (١) - كتاب الصلاة 📎 [ https://t.me/daririhasan/4350 ] * الدرس (٢) - كتاب الصلاة 📎 [ https://t.me/daririhasan/4352 ] * الدرس (٣) - كتاب الصلاة 📎 [ https://t.me/daririhasan/4366 ] * الدرس (٤) - كتاب الصلاة 📎 [ https://t.me/daririh</t>
+          <t>مقال بعنوان الذكاء الاصطناعي ، ومواقع التواصل الاجتماعي بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : معاشر القراء الكرام : إنَّ نعمة الجوالات الحديثة ، وأجهزة الحاسب الآلي نعمةٌ عظيمة إذا استخدمت فيما ينف</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -36282,11 +35466,11 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>message6987</t>
+          <t>message7200</t>
         </is>
       </c>
       <c r="I235" t="n">
-        <v>4193</v>
+        <v>4081</v>
       </c>
       <c r="J235" t="inlineStr">
         <is>
@@ -36305,7 +35489,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>11.05.2026</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -36315,12 +35499,12 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>فهرس دروس فتاوى أركان الإسلام</t>
+          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِنْدَ اللَّهِ عَظِيمٌ – النور : 15 وقال صلى الله عليه وسلـم : – كَفَى بِالْمَرْءِ كَذِبًا أَنْ يُحَدِّثَ بِكُلِّ مَا سمع – رَوَاهُ مُسلم ؛ نسأل الله أن يديم علينا نعمه الظاهرة والباطنة ، وأن يوزعنا ذكرها وشكرها ، ومنها نعمة الجوالات والحاسوبات ، وما فيها من برامج ؛ وتقنيات نافعةٍ ؛ لخدمة الدين ، ثمَّ المليك ، والوطن .</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t xml:space="preserve">فهرس دروس فتاوى أركان الإسلام 3/3 * الدرس (٦٧) - كتاب الصلاة 📎 [ https://t.me/daririhasan/5499 ] * الدرس (٦٨) - كتاب الصلاة 📎 [ https://t.me/daririhasan/5511 ] * الدرس (١) - كتاب الحج 📎 [ https://t.me/daririhasan/4410 ] * الدرس (٢) - كتاب الحج 📎 [ https://t.me/daririhasan/4422 ] </t>
+          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِن</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -36330,11 +35514,11 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>message6988</t>
+          <t>message7201</t>
         </is>
       </c>
       <c r="I236" t="n">
-        <v>1439</v>
+        <v>1062</v>
       </c>
       <c r="J236" t="inlineStr">
         <is>
@@ -36353,7 +35537,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>15.04.2026</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -36363,12 +35547,12 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>فهرس دروس القول السديد شرح كتاب التوحيد</t>
+          <t>جديد 💥</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>📚 فهرس دروس القول السديد شرح كتاب التوحيد ━━━━━━━━━━━━━━━━━━━━━━ 🎙 مع فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ ━━━━━━━━━━━━━━━━━━━━━━ الدرس رقم ١ 📎 [ https://t.me/daririhasan/4678 ] الدرس رقم ٢ 📎 https://t.me/daririhasan/4709 ] الدرس رقم ٣ 📎 [ https://t.me/da</t>
+          <t xml:space="preserve">💥جديد 💥 📖 { العِلْمُ أشْرَفُ مَطْلُوبٍ وَطَالِبُهُ للهِ أكْرَمُ مَن يَمْشِي عَلى قَدَمِ } 📚 🎙️( تم التسجيل- بحمدالله تعالى )🔊 📌 [ الدروس العلمية ]📚 📌" لشهر- شوال " 1447/10/26هجري 🌱 📋 " اسبوعياً " كل يوم الثلاثاء ✅ 🕣 بعد صلاة العشاء👇 📡《عن بُعد 》📡 📚 شرح كتاب- [ معارج القبول في شرح </t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -36378,15 +35562,15 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>message6989</t>
+          <t>message6787</t>
         </is>
       </c>
       <c r="I237" t="n">
-        <v>777</v>
+        <v>772</v>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>messages_june1.html</t>
+          <t>messages_new.html</t>
         </is>
       </c>
     </row>
@@ -36401,7 +35585,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>17.04.2026</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -36411,12 +35595,12 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>فهرس خطبة الجمعة</t>
+          <t>ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!»</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 1 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ١) صفة صلاة النبي ﷺ | ٢٤ جمادى الآخرة ١٤٣٨هـ 📎 https://t.me/daririhasan/80 ٢) سيرة الإمام زيد بن محمد المدخلي | ٢٤ جمادى الآخرة ١٤٣٨هـ 📎 https://t.me/daririhas</t>
+          <t>#فوائد ♦|«ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله- : «وإنَّ ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة، والاستهانة بهم؛ لأن هذا ممَّا يُس</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -36426,15 +35610,15 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>message6999</t>
+          <t>message6817</t>
         </is>
       </c>
       <c r="I238" t="n">
-        <v>4015</v>
+        <v>936</v>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>messages_june1.html</t>
+          <t>messages_new.html</t>
         </is>
       </c>
     </row>
@@ -36449,7 +35633,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>30.04.2026</t>
+          <t>17.04.2026</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -36459,12 +35643,12 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>فهرس خطبة الجمعة</t>
+          <t>يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!»</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t xml:space="preserve">📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 2 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٥١) من أحكام النكاح ٢ | ١٥ ربيع الأول ١٤٤١هـ 📎 https://t.me/daririhasan/496 ٥٢) من أحكام النكاح ٣ | ١٥ ربيع الأول ١٤٤١هـ 📎 https://t.me/daririhasan/497 ٥٣) من </t>
+          <t xml:space="preserve">#فوائد ♦|«يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله-: «فالمهم أنَّ الدعوة يبدأ فيها بالأهم فالمهم، وأنَّ الدعوة إلى التوحيد لمن أهم المهمات؛ يجب عليك أن تُنصِّص على </t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -36474,829 +35658,13 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>message7000</t>
+          <t>message6820</t>
         </is>
       </c>
       <c r="I239" t="n">
-        <v>4026</v>
+        <v>1318</v>
       </c>
       <c r="J239" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="n">
-        <v>381</v>
-      </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C240" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F240" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 3 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٩٨) جماعة الإخوان المسلمين | ٦ ربيع الثاني ١٤٤٢هـ 📎 https://t.me/daririhasan/1301 ٩٩) رزق الله تعالى لعباده | ١٢ ربيع الثاني ١٤٤٢هـ 📎 https://t.me/daririhasan/</t>
-        </is>
-      </c>
-      <c r="G240" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H240" t="inlineStr">
-        <is>
-          <t>message7001</t>
-        </is>
-      </c>
-      <c r="I240" t="n">
-        <v>4034</v>
-      </c>
-      <c r="J240" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="n">
-        <v>382</v>
-      </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F241" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 4 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ١٤٥) عبد الرحمن بن عوف رضي الله عنه | ٢٠ ذو الحجة ١٤٤٢هـ 📎 https://t.me/daririhasan/1690 ١٤٦) نهاية العام والأخذ بالاحترازات ضد كورونا | ٢٧ ذو الحجة ١٤٤٢هـ 📎 h</t>
-        </is>
-      </c>
-      <c r="G241" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H241" t="inlineStr">
-        <is>
-          <t>message7002</t>
-        </is>
-      </c>
-      <c r="I241" t="n">
-        <v>4014</v>
-      </c>
-      <c r="J241" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="n">
-        <v>383</v>
-      </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F242" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 5 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ١٩١) من أحكام الأضحية | ٥ ذو الحجة ١٤٤٣هـ 📎 https://t.me/daririhasan/2280 ١٩٢) أفضل أيام العام | ٩ ذو الحجة ١٤٤٣هـ 📎 https://t.me/daririhasan/2288 ١٩٣) المدينة</t>
-        </is>
-      </c>
-      <c r="G242" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H242" t="inlineStr">
-        <is>
-          <t>message7003</t>
-        </is>
-      </c>
-      <c r="I242" t="n">
-        <v>4019</v>
-      </c>
-      <c r="J242" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="n">
-        <v>384</v>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F243" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 6 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٢٣٦) قصة موسى عليه السلام (٧) | ٦ ذو القعدة ١٤٤٤هـ 📎 https://t.me/daririhasan/3328 ٢٣٧) قصة موسى عليه السلام (٨) | ١٣ ذو القعدة ١٤٤٤هـ 📎 https://t.me/daririhas</t>
-        </is>
-      </c>
-      <c r="G243" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H243" t="inlineStr">
-        <is>
-          <t>message7004</t>
-        </is>
-      </c>
-      <c r="I243" t="n">
-        <v>3953</v>
-      </c>
-      <c r="J243" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="n">
-        <v>385</v>
-      </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D244" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>فهرس خطبة الجمعة</t>
-        </is>
-      </c>
-      <c r="F244" t="inlineStr">
-        <is>
-          <t>📚 فهرس خطبة الجمعة 🎙 فضيلة الشيخ حسن بن محمد منصور الدغريري ━━━━━━━━━━━━━━━━━━━━━━ 📩 رسالة 7 من 8 ━━━━━━━━━━━━━━━━━━━━━━ ٢٨٢) الأعمال الصالحة في العشر والأخذ بأسباب السلامة في الحج | ١ ذو الحجة ١٤٤٥هـ 📎 https://t.me/daririhasan/4449 ٢٨٣) صفة الأنساك الثلاثة (٢) | ١٢ ذو الحجة ١٤٤٥</t>
-        </is>
-      </c>
-      <c r="G244" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H244" t="inlineStr">
-        <is>
-          <t>message7005</t>
-        </is>
-      </c>
-      <c r="I244" t="n">
-        <v>3958</v>
-      </c>
-      <c r="J244" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="n">
-        <v>386</v>
-      </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D245" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>فهرس دروس الأفنان الندية شرح السبل السوية في فقه السنن المروية للشيخ العلامة زيد المدخلي رحمه الله</t>
-        </is>
-      </c>
-      <c r="F245" t="inlineStr">
-        <is>
-          <t>📍فهرس دروس الأفنان الندية شرح السبل السوية في فقه السنن المروية للشيخ العلامة زيد المدخلي رحمه الله 🎙️لفضيلة الشيخ حسن الدغريري حفظه الله 🔹فهرس الدروس : 🔸 كتاب الطهارة - الدرس الأول 📎 https://t.me/daririhasan/2371 - الدرس الثاني 📎 https://t.me/daririhasan/2392 - الدرس الثالث 📎 ht</t>
-        </is>
-      </c>
-      <c r="G245" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H245" t="inlineStr">
-        <is>
-          <t>message7008</t>
-        </is>
-      </c>
-      <c r="I245" t="n">
-        <v>4062</v>
-      </c>
-      <c r="J245" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="n">
-        <v>387</v>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>30.04.2026</t>
-        </is>
-      </c>
-      <c r="D246" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>كتاب البيوع</t>
-        </is>
-      </c>
-      <c r="F246" t="inlineStr">
-        <is>
-          <t>🔸كتاب البيوع - الدرس الأول 📎 https://t.me/daririhasan/5103 - الدرس الثاني 📎 https://t.me/daririhasan/5122 - الدرس الثالث 📎 https://t.me/daririhasan/5134 الدرس الرابع 📎 https://t.me/daririhasan/5158 - الدرس الخامس 📎 https://t.me/daririhasan/5538 - الدرس السادس 📎 https://t.me/darir</t>
-        </is>
-      </c>
-      <c r="G246" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H246" t="inlineStr">
-        <is>
-          <t>message7010</t>
-        </is>
-      </c>
-      <c r="I246" t="n">
-        <v>2562</v>
-      </c>
-      <c r="J246" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="n">
-        <v>388</v>
-      </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>09.05.2026</t>
-        </is>
-      </c>
-      <c r="D247" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
-        </is>
-      </c>
-      <c r="F247" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وأخيراً : فهذه هي الصوفية، وهذه عقيدتها، إيمان بالمادة، وكفر بالله، إيمان بالكشف الشيطاني للشيوخ، وكفر بالقرآن، تصديق للخرافة، وجُحُودٌ للتوحيد، انغماس في البدع، ورفض للسنن، إيمان بالباطل، وكفر بالحق، تطاول عَلَى عظمة الله وألوهيته، وادعاء</t>
-        </is>
-      </c>
-      <c r="G247" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H247" t="inlineStr">
-        <is>
-          <t>message7162</t>
-        </is>
-      </c>
-      <c r="I247" t="n">
-        <v>576</v>
-      </c>
-      <c r="J247" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="n">
-        <v>389</v>
-      </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>09.05.2026</t>
-        </is>
-      </c>
-      <c r="D248" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E248" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله:</t>
-        </is>
-      </c>
-      <c r="F248" t="inlineStr">
-        <is>
-          <t>قال الشيخ أحمد بن يحيى النجمي رحمه الله: وكذلك قوله: ولا صَفَرَ »؛ فإن أهل الجاهلية كانوا يتشاءمون بشهر صفر، فأخبر النبي ﷺ أَنَّ الشهر لا شؤم فيه، بل هو كسائر الشهور، وَقَدْ كان لناس أيضا يتشاءمون ببعض الأيام كيوم الأربعاء من آخر كل شهر، ويُسمونه ربوعا لم يدور، ويعتقدون فيه أنه ي</t>
-        </is>
-      </c>
-      <c r="G248" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H248" t="inlineStr">
-        <is>
-          <t>message7177</t>
-        </is>
-      </c>
-      <c r="I248" t="n">
-        <v>484</v>
-      </c>
-      <c r="J248" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="n">
-        <v>390</v>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>10.05.2026</t>
-        </is>
-      </c>
-      <c r="D249" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E249" t="inlineStr">
-        <is>
-          <t>مقال بعنوان</t>
-        </is>
-      </c>
-      <c r="F249" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مقال بعنوان الشيخ العلامة / ناصر بن أحمد جبران قحل رحمه الله ( 1361 هـ-1447هـ ) بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : أخواني القراء الفضلاء : لقد رحل صباح يوم الثلاثاء ١٨ / ١١ / ١٤٤٧ الشيخ العلامة </t>
-        </is>
-      </c>
-      <c r="G249" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H249" t="inlineStr">
-        <is>
-          <t>message7186</t>
-        </is>
-      </c>
-      <c r="I249" t="n">
-        <v>3978</v>
-      </c>
-      <c r="J249" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="n">
-        <v>391</v>
-      </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>10.05.2026</t>
-        </is>
-      </c>
-      <c r="D250" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ فنظموا فيه شعراً ، وكتبوا فيه نثراً على جهده وجهاده في طلب العلم ، ونشره ، ولولا خشية الاطالة في هذا المقال لذكرت لكم بعضها ؛ وعزاؤنا في طلابه أن ينشروا علمه بين الأنام ، وسيرته الطيبة بين الناس ، ونسأل الله أن يجعل ما تركه من مقاطع صوتية نافعةٍ ، ودروس علمية مسجلة ، وتلاواتٍ قرآنية مجودة نديةٍ ، وسيرةٍ مباركةٍ مؤثرةٍ ، وعملٍ صالحٍ دلَّ عليه ، وأخلاقٍ وآدابٍ حسنةٍ تخلَّق بها ، ومريضٍ بالسحر أو غيره قد تسبب في شفائه في ميزان حسناته يوم تخف الموازين ، وأن يجمعنا به ، وبالنبيين ، والشهداء ، والصالحين ، وسائر العلماء الناصحين في جنات النعيم ، وأن يقينا جميعاً عذاب القبر والجحيم . اللهم آمين .</t>
-        </is>
-      </c>
-      <c r="F250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">أخي القارئ الفاضل : من تتلمذ على يد هذه الكوكبة النيرة من المشايخ والعلماء ؛ كيف تكون حصيلته اللغوية ، واستفادته الشرعية ؟ لاشكَّ أنَّه قد استفاد منهم علماً جمَّاً ؛ مما جعله من مصافِّ أهل العلم الشرعي ، ومبرزاً فيها ، وقد حزن الناس لوفاة الشيخ ناصر بن أحمد جبران قحل رحمه الله ؛ </t>
-        </is>
-      </c>
-      <c r="G250" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H250" t="inlineStr">
-        <is>
-          <t>message7187</t>
-        </is>
-      </c>
-      <c r="I250" t="n">
-        <v>875</v>
-      </c>
-      <c r="J250" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="n">
-        <v>392</v>
-      </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>11.05.2026</t>
-        </is>
-      </c>
-      <c r="D251" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>مقال بعنوان</t>
-        </is>
-      </c>
-      <c r="F251" t="inlineStr">
-        <is>
-          <t>مقال بعنوان الذكاء الاصطناعي ، ومواقع التواصل الاجتماعي بقلم فضيلة الشيخ حسن بن محمد منصور مخزم الدغريري الحمد لله ، والصلاة ، والسلام على رسول الله ، وعلى آله ، وصحبه ، وبعد : معاشر القراء الكرام : إنَّ نعمة الجوالات الحديثة ، وأجهزة الحاسب الآلي نعمةٌ عظيمة إذا استخدمت فيما ينف</t>
-        </is>
-      </c>
-      <c r="G251" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H251" t="inlineStr">
-        <is>
-          <t>message7200</t>
-        </is>
-      </c>
-      <c r="I251" t="n">
-        <v>4081</v>
-      </c>
-      <c r="J251" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="n">
-        <v>393</v>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>11.05.2026</t>
-        </is>
-      </c>
-      <c r="D252" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِنْدَ اللَّهِ عَظِيمٌ – النور : 15 وقال صلى الله عليه وسلـم : – كَفَى بِالْمَرْءِ كَذِبًا أَنْ يُحَدِّثَ بِكُلِّ مَا سمع – رَوَاهُ مُسلم ؛ نسأل الله أن يديم علينا نعمه الظاهرة والباطنة ، وأن يوزعنا ذكرها وشكرها ، ومنها نعمة الجوالات والحاسوبات ، وما فيها من برامج ؛ وتقنيات نافعةٍ ؛ لخدمة الدين ، ثمَّ المليك ، والوطن .</t>
-        </is>
-      </c>
-      <c r="F252" t="inlineStr">
-        <is>
-          <t>جَاءَكُمْ فَاسِقٌ بِنَبَإٍ فَتَبَيَّنُوا أَنْ تُصِيبُوا قَوْمًا بِجَهَالَةٍ فَتُصْبِحُوا عَلَى مَا فَعَلْتُمْ نَادِمِينَ – الحجرات : 6 وقال تعالى : – إِذْ تَلَقَّوْنَهُ بِأَلْسِنَتِكُمْ وَتَقُولُونَ بِأَفْوَاهِكُمْ مَا لَيْسَ لَكُمْ بِهِ عِلْمٌ وَتَحْسَبُونَهُ هَيِّنًا وَهُوَ عِن</t>
-        </is>
-      </c>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H252" t="inlineStr">
-        <is>
-          <t>message7201</t>
-        </is>
-      </c>
-      <c r="I252" t="n">
-        <v>1062</v>
-      </c>
-      <c r="J252" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="n">
-        <v>394</v>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>21.05.2026</t>
-        </is>
-      </c>
-      <c r="D253" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>فهرس دروس</t>
-        </is>
-      </c>
-      <c r="F253" t="inlineStr">
-        <is>
-          <t>فهرس دروس #التعليق_على_كتاب_الأربعين_النووية 🎙 للشيخ الفاضل: #حسن_بن_محمد_الدغريري -الدرس الأول 📎 https://t.me/daririhasan/705 -الدرس الثاني 📎 https://t.me/daririhasan/708 -الدرس الثالث 📎 https://t.me/daririhasan/709 -الدرس الرابع 📎 https://t.me/daririhasan/717 -الدرس الخامس 📎 ht</t>
-        </is>
-      </c>
-      <c r="G253" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H253" t="inlineStr">
-        <is>
-          <t>message7423</t>
-        </is>
-      </c>
-      <c r="I253" t="n">
-        <v>2391</v>
-      </c>
-      <c r="J253" t="inlineStr">
-        <is>
-          <t>messages_june1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="n">
-        <v>395</v>
-      </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>15.04.2026</t>
-        </is>
-      </c>
-      <c r="D254" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>جديد 💥</t>
-        </is>
-      </c>
-      <c r="F254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">💥جديد 💥 📖 { العِلْمُ أشْرَفُ مَطْلُوبٍ وَطَالِبُهُ للهِ أكْرَمُ مَن يَمْشِي عَلى قَدَمِ } 📚 🎙️( تم التسجيل- بحمدالله تعالى )🔊 📌 [ الدروس العلمية ]📚 📌" لشهر- شوال " 1447/10/26هجري 🌱 📋 " اسبوعياً " كل يوم الثلاثاء ✅ 🕣 بعد صلاة العشاء👇 📡《عن بُعد 》📡 📚 شرح كتاب- [ معارج القبول في شرح </t>
-        </is>
-      </c>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H254" t="inlineStr">
-        <is>
-          <t>message6787</t>
-        </is>
-      </c>
-      <c r="I254" t="n">
-        <v>772</v>
-      </c>
-      <c r="J254" t="inlineStr">
-        <is>
-          <t>messages_new.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="n">
-        <v>396</v>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
-      </c>
-      <c r="D255" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!»</t>
-        </is>
-      </c>
-      <c r="F255" t="inlineStr">
-        <is>
-          <t>#فوائد ♦|«ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله- : «وإنَّ ممَّا يُعدُّ من الخروج: ذكر مثالب الولاة، والطعن فيهم، والإنكار عليهم بين الجموع الحاشدة، والاستهانة بهم؛ لأن هذا ممَّا يُس</t>
-        </is>
-      </c>
-      <c r="G255" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H255" t="inlineStr">
-        <is>
-          <t>message6817</t>
-        </is>
-      </c>
-      <c r="I255" t="n">
-        <v>936</v>
-      </c>
-      <c r="J255" t="inlineStr">
-        <is>
-          <t>messages_new.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="n">
-        <v>397</v>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>TelegramArticle</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
-      </c>
-      <c r="D256" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!»</t>
-        </is>
-      </c>
-      <c r="F256" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#فوائد ♦|«يجب عليك أن تُنصِّص عليهم، وأن تبين حالهم، فلا تخشى منهم، والله سُبْحَانَهُ وَتَعَالَى يرضى عنك إذا قلت الحق!» ○ يقول العلامة أحمد بن يحيى النجمي -رحمه الله-: «فالمهم أنَّ الدعوة يبدأ فيها بالأهم فالمهم، وأنَّ الدعوة إلى التوحيد لمن أهم المهمات؛ يجب عليك أن تُنصِّص على </t>
-        </is>
-      </c>
-      <c r="G256" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H256" t="inlineStr">
-        <is>
-          <t>message6820</t>
-        </is>
-      </c>
-      <c r="I256" t="n">
-        <v>1318</v>
-      </c>
-      <c r="J256" t="inlineStr">
         <is>
           <t>messages_new.html</t>
         </is>
@@ -37313,7 +35681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37344,32 +35712,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>DupReason</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>FetchStatus</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
           <t>MessageID</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>FullTextChars</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>SourceFile</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>DupReason</t>
         </is>
       </c>
     </row>
@@ -37399,30 +35747,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>••• ═══ ༻✿༺═══ ••• (❓) سائل يقول : السلام عليكم ورحمه الله وبركاته حياكم شيخنا نريد منكم نصيحة للمسلمين في رمضان وجزاكم الله خيرا 🔹الجواب : نصيحتي لهم أن يتقوا الله ويعظِّموا شهر رمضان بفعل الأعمال الصالحة المشروعة فيه من الصِّيام والقيام والصَّدقة وتلاوة القرآن وسائر الأعمال الص</t>
+          <t>duplicate content</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>message2131</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>585</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>messages2.html</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>duplicate content</t>
         </is>
       </c>
     </row>
@@ -37452,30 +35782,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">•••••✦✦✦✿✿✿✦✦✦••••• #فوائد قال شيخنا حسن بن محمد منصور الدغريري -حفظه الله- : ‏❍ «...فلذلك أيها الإخوة يجب علينا أن نطلب العلم. لأن طلب العلم الشرعي فريضة على كل مسلم ومسلمة، لأن بتركه تحصل البدعة ويحصل الكفر ويحصل الشرك ويحصل الضلال، فما كان واجبا لا بد من آدائه، ولا يتم الواجب </t>
+          <t>duplicate content</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>message2812</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>536</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>messages2.html</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>duplicate content</t>
         </is>
       </c>
     </row>
@@ -37505,30 +35817,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>•••••✦✦✦✿✿✿✦✦✦••••• #فوائد قال شيخنا حسن الدغريري حفظه الله : ❍‏ عباد الله : علينا أن نحرص على الإكثار من صيام أيام شهر شعبان حتى إذا ما أتى شهر رمضان يكون المسلم قد اعتاد على عبادة الصيام في شهر رمضان الذي أوجب الله صيامه وقد كان من هدي نبينا محمد ﷺ الإكثار من صيام أيام شهر شعبا</t>
+          <t>duplicate content</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>message3036</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>685</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>messages2.html</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>duplicate content</t>
         </is>
       </c>
     </row>
@@ -37558,30 +35852,607 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>*{{📚📚مكتمل📚📚}}* *🔺🔺🔺تـنـبـيـه الأنــــام🔺🔺🔺* *عـلىٰ مـا فـي كتـاب سـبـل السـلام* *مـن الفـوائـد والأحـــكـام* *لفضيلة الشيخ العلامة* * أحمد بن يحيىٰ النجمي* *رحمه الله* *🔺المجلد الأول 📔 https://alnajmi.net/portal/wp-content/uploads/2023/03/talanam1.pdf *🔺 المجلد الثاني 📔 https://</t>
+          <t>duplicate content</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
           <t>message3379</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>985</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>messages2.html</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>duplicate content</t>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>28.01.2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>فهرسة دروس لشروحات وتعليقات على #كتابالصيام |</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>message6309</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>فهرس دروس معارج القبول شرح سلم الوصول للحافظ الحكمي رحمه</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>message6971</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>فهرس دروس شرح كتاب الفقه الميسر</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>message6984</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>فهرس دروس شرح كتاب الفقه الميسر</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>message6985</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>فهرس دروس فتاوى أركان الإسلام</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>message6986</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>فهرس دروس فتاوى أركان الإسلام</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>message6987</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>فهرس دروس فتاوى أركان الإسلام</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>message6988</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>فهرس دروس القول السديد شرح كتاب التوحيد</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>message6989</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>فهرس خطبة الجمعة</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>message6999</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>فهرس خطبة الجمعة</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>message7000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>فهرس خطبة الجمعة</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>message7001</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>فهرس خطبة الجمعة</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>message7002</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>فهرس خطبة الجمعة</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>message7003</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>فهرس خطبة الجمعة</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>message7004</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>فهرس خطبة الجمعة</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>message7005</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>30.04.2026</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>فهرس دروس الأفنان الندية شرح السبل السوية في فقه السنن المروية للشيخ العلامة زيد المدخلي رحمه الله</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>message7008</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TelegramArticle</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>21.05.2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>فهرس دروس</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>فهرس (lesson index, not an article)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>message7423</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Telegram post URLs for all TelegramArticle entries
Each TelegramArticle now has a url field: https://t.me/daririhasan/{msg_number}
All 239 TelegramArticle entries updated.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01An4PrSA3PECn9RaetfjGkW
</commit_message>
<xml_diff>
--- a/output/articles/articles_summary.xlsx
+++ b/output/articles/articles_summary.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All (unique)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asdaa (99)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TGArticles" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TGArticles (239)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/82</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/120</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/181</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/247</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/255</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5083,7 +5083,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/322</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/323</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/324</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/325</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/326</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5323,7 +5323,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/331</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/334</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/336</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/337</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/338</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/339</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/357</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/367</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5707,7 +5707,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/368</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5755,7 +5755,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/381</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/400</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/401</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/402</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/404</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5995,7 +5995,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/407</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6043,7 +6043,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/408</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/409</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6139,7 +6139,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/413</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/423</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/425</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/426</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/427</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/431</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/439</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/444</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6523,7 +6523,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/445</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/446</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/448</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/453</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6715,7 +6715,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/479</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/488</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/494</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6859,7 +6859,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/506</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6907,7 +6907,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/509</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6955,7 +6955,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/512</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -7003,7 +7003,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/514</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/527</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/528</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/544</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/545</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -7243,7 +7243,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/553</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/558</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -7339,7 +7339,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/575</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/596</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/633</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/634</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/635</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/636</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/637</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/642</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -7723,7 +7723,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/647</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/655</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -7819,7 +7819,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/664</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -7867,7 +7867,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/673</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -7915,7 +7915,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/675</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -7963,7 +7963,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/690</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/701</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -8059,7 +8059,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/753</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/772</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/775</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -8203,7 +8203,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/780</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/792</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/794</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/795</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -8395,7 +8395,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/798</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -8443,7 +8443,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/806</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -8491,7 +8491,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/807</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -8539,7 +8539,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/824</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/837</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -8635,7 +8635,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/839</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/896</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/987</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1039</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1046</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -8875,7 +8875,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1053</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -8923,7 +8923,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1060</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1070</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -9019,7 +9019,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1071</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1079</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1093</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -9163,7 +9163,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1094</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1095</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1102</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1116</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1130</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -9403,7 +9403,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1131</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -9451,7 +9451,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1144</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -9499,7 +9499,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1157</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -9547,7 +9547,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1171</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -9595,7 +9595,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1178</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -9643,7 +9643,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1190</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1206</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1209</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1265</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -9835,7 +9835,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1286</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1350</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -9931,7 +9931,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1399</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1402</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -10027,7 +10027,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1419</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -10075,7 +10075,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1439</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -10123,7 +10123,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1440</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -10171,7 +10171,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1463</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -10219,7 +10219,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1478</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1479</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -10315,7 +10315,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1484</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -10363,7 +10363,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1494</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1498</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -10459,7 +10459,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1500</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -10507,7 +10507,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1508</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -10555,7 +10555,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1542</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -10603,7 +10603,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1558</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1691</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -10699,7 +10699,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1703</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -10747,7 +10747,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1704</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1705</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1728</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -10891,7 +10891,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1771</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1773</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -10987,7 +10987,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1874</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -11035,7 +11035,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1875</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1879</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -11131,7 +11131,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1894</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1914</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -11227,7 +11227,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2004</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -11275,7 +11275,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2070</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2072</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2073</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -11419,7 +11419,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2074</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2099</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -11515,7 +11515,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2159</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -11563,7 +11563,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2162</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -11611,7 +11611,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2172</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -11659,7 +11659,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2201</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
@@ -11707,7 +11707,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2222</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
@@ -11755,7 +11755,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2234</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2342</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -11851,7 +11851,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2345</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -11899,7 +11899,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2353</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2536</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2561</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2576</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -12091,7 +12091,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2577</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -12139,7 +12139,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2656</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2724</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -12235,7 +12235,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2758</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -12283,7 +12283,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2781</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -12331,7 +12331,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2842</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -12379,7 +12379,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2853</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -12427,7 +12427,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2856</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -12475,7 +12475,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2888</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -12523,7 +12523,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2912</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -12571,7 +12571,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2913</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -12619,7 +12619,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2969</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3005</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -12715,7 +12715,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3084</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -12763,7 +12763,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3175</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -12811,7 +12811,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3188</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -12859,7 +12859,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3223</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3226</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -12955,7 +12955,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3446</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
@@ -13003,7 +13003,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3465</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3467</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -13099,7 +13099,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3469</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -13147,7 +13147,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3730</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
@@ -13195,7 +13195,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3792</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -13243,7 +13243,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3962</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
@@ -13291,7 +13291,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3969</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -13339,7 +13339,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4013</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4075</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4300</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4329</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -13531,7 +13531,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4336</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -13579,7 +13579,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4339</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -13627,7 +13627,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4341</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -13675,7 +13675,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4364</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -13723,7 +13723,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4377</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -13771,7 +13771,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4405</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -13819,7 +13819,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4496</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -13867,7 +13867,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4691</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -13915,7 +13915,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4735</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -13963,7 +13963,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4875</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -14011,7 +14011,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4918</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -14059,7 +14059,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4934</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4935</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -14155,7 +14155,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4937</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -14203,7 +14203,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4942</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -14251,7 +14251,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5033</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -14299,7 +14299,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5035</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -14347,7 +14347,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5037</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5039</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -14443,7 +14443,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5080</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -14491,7 +14491,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5145</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -14539,7 +14539,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5146</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -14587,7 +14587,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5241</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -14635,7 +14635,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5286</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -14683,7 +14683,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5290</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -14731,7 +14731,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5292</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -14779,7 +14779,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5359</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -14827,7 +14827,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5411</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -14875,7 +14875,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5417</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -14923,7 +14923,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5504</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -14971,7 +14971,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5531</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5632</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5663</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -15115,7 +15115,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5691</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -15163,7 +15163,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5697</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -15211,7 +15211,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5698</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5834</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -15307,7 +15307,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5898</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -15355,7 +15355,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6042</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -15403,7 +15403,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6180</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -15451,7 +15451,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6183</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -15499,7 +15499,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6199</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -15547,7 +15547,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6444</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -15595,7 +15595,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6552</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -15643,7 +15643,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6557</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -15691,7 +15691,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6617</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -15739,7 +15739,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6904</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -15787,7 +15787,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7010</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -15835,7 +15835,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7162</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -15883,7 +15883,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7177</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -15931,7 +15931,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7186</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -15979,7 +15979,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7187</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -16027,7 +16027,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7200</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -16075,7 +16075,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7201</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -16123,7 +16123,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6787</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -16171,7 +16171,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6817</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -16219,7 +16219,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6820</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5465</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -20803,7 +20803,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/82</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -20851,7 +20851,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/120</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -20899,7 +20899,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/181</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -20947,7 +20947,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/247</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -20995,7 +20995,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/255</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -21043,7 +21043,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/322</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -21091,7 +21091,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/323</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -21139,7 +21139,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/324</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -21187,7 +21187,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/325</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -21235,7 +21235,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/326</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -21283,7 +21283,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/331</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -21331,7 +21331,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/334</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -21379,7 +21379,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/336</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -21427,7 +21427,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/337</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -21475,7 +21475,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/338</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -21523,7 +21523,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/339</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -21571,7 +21571,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/357</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -21619,7 +21619,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/367</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -21667,7 +21667,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/368</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -21715,7 +21715,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/381</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -21763,7 +21763,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/400</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -21811,7 +21811,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/401</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -21859,7 +21859,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/402</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -21907,7 +21907,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/404</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -21955,7 +21955,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/407</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -22003,7 +22003,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/408</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -22051,7 +22051,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/409</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -22099,7 +22099,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/413</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -22147,7 +22147,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/423</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -22195,7 +22195,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/425</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -22243,7 +22243,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/426</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -22291,7 +22291,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/427</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -22339,7 +22339,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/431</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -22387,7 +22387,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/439</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -22435,7 +22435,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/444</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -22483,7 +22483,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/445</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -22531,7 +22531,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/446</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -22579,7 +22579,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/448</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -22627,7 +22627,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/453</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -22675,7 +22675,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/479</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -22723,7 +22723,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/488</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -22771,7 +22771,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/494</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -22819,7 +22819,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/506</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -22867,7 +22867,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/509</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -22915,7 +22915,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/512</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -22963,7 +22963,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/514</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -23011,7 +23011,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/527</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -23059,7 +23059,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/528</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/544</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -23155,7 +23155,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/545</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -23203,7 +23203,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/553</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -23251,7 +23251,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/558</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -23299,7 +23299,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/575</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -23347,7 +23347,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/596</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -23395,7 +23395,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/633</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -23443,7 +23443,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/634</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -23491,7 +23491,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/635</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -23539,7 +23539,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/636</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -23587,7 +23587,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/637</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -23635,7 +23635,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/642</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -23683,7 +23683,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/647</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -23731,7 +23731,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/655</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -23779,7 +23779,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/664</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -23827,7 +23827,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/673</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -23875,7 +23875,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/675</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -23923,7 +23923,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/690</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -23971,7 +23971,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/701</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -24019,7 +24019,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/753</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -24067,7 +24067,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/772</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -24115,7 +24115,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/775</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -24163,7 +24163,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/780</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -24211,7 +24211,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/792</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -24259,7 +24259,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/794</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -24307,7 +24307,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/795</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -24355,7 +24355,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/798</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -24403,7 +24403,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/806</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -24451,7 +24451,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/807</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -24499,7 +24499,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/824</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -24547,7 +24547,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/837</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -24595,7 +24595,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/839</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -24643,7 +24643,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/896</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -24691,7 +24691,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/987</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -24739,7 +24739,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1039</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -24787,7 +24787,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1046</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -24835,7 +24835,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1053</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -24883,7 +24883,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1060</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -24931,7 +24931,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1070</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -24979,7 +24979,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1071</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -25027,7 +25027,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1079</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -25075,7 +25075,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1093</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -25123,7 +25123,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1094</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -25171,7 +25171,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1095</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -25219,7 +25219,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1102</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -25267,7 +25267,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1116</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -25315,7 +25315,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1130</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -25363,7 +25363,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1131</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -25411,7 +25411,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1144</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -25459,7 +25459,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1157</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -25507,7 +25507,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1171</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -25555,7 +25555,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1178</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -25603,7 +25603,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1190</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -25651,7 +25651,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1206</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -25699,7 +25699,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1209</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -25747,7 +25747,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1265</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -25795,7 +25795,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1286</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -25843,7 +25843,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1350</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -25891,7 +25891,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1399</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -25939,7 +25939,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1402</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -25987,7 +25987,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1419</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -26035,7 +26035,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1439</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -26083,7 +26083,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1440</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -26131,7 +26131,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1463</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -26179,7 +26179,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1478</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -26227,7 +26227,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1479</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -26275,7 +26275,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1484</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -26323,7 +26323,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1494</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -26371,7 +26371,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1498</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -26419,7 +26419,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1500</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -26467,7 +26467,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1508</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -26515,7 +26515,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1542</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -26563,7 +26563,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1558</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -26611,7 +26611,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1691</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -26659,7 +26659,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1703</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -26707,7 +26707,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1704</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -26755,7 +26755,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1705</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -26803,7 +26803,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1728</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -26851,7 +26851,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1771</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -26899,7 +26899,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1773</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -26947,7 +26947,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1874</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -26995,7 +26995,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1875</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -27043,7 +27043,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1879</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -27091,7 +27091,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1894</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -27139,7 +27139,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/1914</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -27187,7 +27187,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2004</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -27235,7 +27235,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2070</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -27283,7 +27283,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2072</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -27331,7 +27331,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2073</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -27379,7 +27379,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2074</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -27427,7 +27427,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2099</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -27475,7 +27475,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2159</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2162</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -27571,7 +27571,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2172</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -27619,7 +27619,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2201</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -27667,7 +27667,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2222</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -27715,7 +27715,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2234</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -27763,7 +27763,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2342</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -27811,7 +27811,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2345</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -27859,7 +27859,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2353</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -27907,7 +27907,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2536</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -27955,7 +27955,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2561</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -28003,7 +28003,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2576</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -28051,7 +28051,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2577</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -28099,7 +28099,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2656</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -28147,7 +28147,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2724</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -28195,7 +28195,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2758</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -28243,7 +28243,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2781</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -28291,7 +28291,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2842</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -28339,7 +28339,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2853</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -28387,7 +28387,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2856</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -28435,7 +28435,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2888</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -28483,7 +28483,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2912</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -28531,7 +28531,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2913</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -28579,7 +28579,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/2969</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -28627,7 +28627,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3005</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -28675,7 +28675,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3084</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -28723,7 +28723,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3175</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -28771,7 +28771,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3188</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -28819,7 +28819,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3223</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -28867,7 +28867,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3226</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -28915,7 +28915,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3446</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -28963,7 +28963,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3465</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -29011,7 +29011,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3467</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -29059,7 +29059,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3469</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -29107,7 +29107,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3730</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -29155,7 +29155,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3792</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -29203,7 +29203,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3962</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -29251,7 +29251,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/3969</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -29299,7 +29299,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4013</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -29347,7 +29347,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4075</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -29395,7 +29395,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4300</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -29443,7 +29443,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4329</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -29491,7 +29491,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4336</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -29539,7 +29539,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4339</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -29587,7 +29587,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4341</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -29635,7 +29635,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4364</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -29683,7 +29683,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4377</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -29731,7 +29731,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4405</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -29779,7 +29779,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4496</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -29827,7 +29827,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4691</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -29875,7 +29875,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4735</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -29923,7 +29923,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4875</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -29971,7 +29971,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4918</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -30019,7 +30019,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4934</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -30067,7 +30067,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4935</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -30115,7 +30115,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4937</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -30163,7 +30163,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/4942</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -30211,7 +30211,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5033</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -30259,7 +30259,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5035</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -30307,7 +30307,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5037</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -30355,7 +30355,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5039</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -30403,7 +30403,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5080</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -30451,7 +30451,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5145</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -30499,7 +30499,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5146</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -30547,7 +30547,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5241</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -30595,7 +30595,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5286</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -30643,7 +30643,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5290</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -30691,7 +30691,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5292</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -30739,7 +30739,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5359</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -30787,7 +30787,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5411</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -30835,7 +30835,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5417</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -30883,7 +30883,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5504</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -30931,7 +30931,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5531</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -30979,7 +30979,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5632</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -31027,7 +31027,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5663</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -31075,7 +31075,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5691</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -31123,7 +31123,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5697</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -31171,7 +31171,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5698</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -31219,7 +31219,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5834</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -31267,7 +31267,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5898</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -31315,7 +31315,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6042</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -31363,7 +31363,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6180</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -31411,7 +31411,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6183</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -31459,7 +31459,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6199</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -31507,7 +31507,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6444</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -31555,7 +31555,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6552</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -31603,7 +31603,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6557</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -31651,7 +31651,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6617</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -31699,7 +31699,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6904</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -31747,7 +31747,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7010</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -31795,7 +31795,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7162</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -31843,7 +31843,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7177</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -31891,7 +31891,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7186</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -31939,7 +31939,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7187</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -31987,7 +31987,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7200</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -32035,7 +32035,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/7201</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -32083,7 +32083,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6787</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -32131,7 +32131,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6817</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -32179,7 +32179,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/6820</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -32227,7 +32227,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://t.me/daririhasan/5465</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">

</xml_diff>